<commit_message>
add updated excel kb
</commit_message>
<xml_diff>
--- a/Excels/Knowledge Base.xlsx
+++ b/Excels/Knowledge Base.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itservicewn.sharepoint.com/sites/VODAFONEVIER/Freigegebene Dokumente/General/FAQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C437004-640A-488E-8379-CFE0609A3568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE63BB4F-29FE-4BDB-B71C-0B8AA884EBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>Zusätzliche Informationen / Wissensdatenbank für den FAQ-Bot</t>
   </si>
@@ -96,30 +96,7 @@
     <t>Einspeiseanlagen – Zählerstand</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Für Einspeiseanlagen ist der Zählerstand mit dem Zählercode </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2.8.0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> relevant. Dieser Wert zeigt die ins Stromnetz eingespeiste Energiemenge an und ist für die Abrechnung der Einspeisevergütung relevant.</t>
-    </r>
+    <t>Für Einspeiseanlagen ist der Zählerstand mit dem Zählercode 2.8.0 relevant. Dieser Wert zeigt die ins Stromnetz eingespeiste Energiemenge an und ist für die Abrechnung der Einspeisevergütung relevant.</t>
   </si>
   <si>
     <t>Freibad Waiblingen – Öffnungszeiten</t>
@@ -128,6 +105,18 @@
     <t>Das Freibad Waiblingen ist jährlich vom 1. Mai bis 15. September geöffnet. Während dieses Zeitraums gelten täglich die Öffnungszeiten von 07:00 Uhr bis 20:00 Uhr.</t>
   </si>
   <si>
+    <t>Freibad Waiblingen - Badeschluss</t>
+  </si>
+  <si>
+    <t>Badeschluss ist im Freibad Waiblingen ist um 19:40 Uhr.</t>
+  </si>
+  <si>
+    <t>Freibad Waiblingen - Ermäßigung Rentner</t>
+  </si>
+  <si>
+    <t>Nein, Rentner erhalten keine Ermäßigung im Freibad Waiblingen.</t>
+  </si>
+  <si>
     <t>Gasversorgung – Belieferung außerhalb des Versorgungsgebiets</t>
   </si>
   <si>
@@ -143,13 +132,13 @@
     <t>Lieferantenwechsel – Widerruf Fremdvertrag</t>
   </si>
   <si>
-    <t>Hat ein Kunde versehentlich oder ungewollt einen Vertrag bei einem anderen Energieversorger abgeschlossen und möchte weiterhin von den Stadtwerken Waiblingen beliefert werden, muss der Vertrag beim anderen Lieferanten widerrufen werden. Dies gilt beispielsweise auch für Verträge, die an der Haustür abgeschlossen wurden oder zu deren Abschluss sich der Kunde überredet fühlte. Für die Prüfung und weitere Bearbeitung durch die Stadtwerke Waiblingen wird die schriftliche Widerrufsbestätigung des anderen Lieferanten benötigt. Der Kunde soll diese Bestätigung per E-Mail an Vertrieb@stadtwerke-waiblingen.de senden. Nach Eingang der Widerrufsbestätigung wird der Vorgang geprüft und bearbeitet.</t>
+    <t>Haben Sie versehentlich oder ungewollt einen Vertrag bei einem anderen Energieversorger abgeschlossen und möchten weiterhin von den Stadtwerken Waiblingen beliefert werden, muss der Vertrag beim anderen Lieferanten widerrufen werden. Dies gilt beispielsweise auch für Verträge, die an der Haustür abgeschlossen wurden oder zu deren Abschluss sich der Kunde überredet fühlte. Für die Prüfung und weitere Bearbeitung durch die Stadtwerke Waiblingen wird die schriftliche Widerrufsbestätigung des anderen Lieferanten benötigt. Der Kunde soll diese Bestätigung per E-Mail an Vertrieb@stadtwerke-waiblingen.de senden. Nach Eingang der Widerrufsbestätigung wird der Vorgang geprüft und bearbeitet.</t>
   </si>
   <si>
     <t>Tarifwechsel – Widerruf</t>
   </si>
   <si>
-    <t>Ein bereits angestoßener Tarifwechsel kann widerrufen werden. Der Widerruf muss schriftlich erfolgen. Hierfür kann der Kunde eine E-Mail an den Vertrieb der Stadtwerke Waiblingen senden oder den Widerrufs-Button auf der Website nutzen. Nach Eingang des Widerrufs wird das Anliegen geprüft und bearbeitet.</t>
+    <t>Ein bereits angestoßener Tarifwechsel kann widerrufen werden. Der Widerruf muss schriftlich erfolgen. Hierfür können Sie eine E-Mail an vertrieb@stadtwerke-waiblingen.de senden oder den Widerrufs-Button auf der Website nutzen. Nach Eingang des Widerrufs wird das Anliegen geprüft und bearbeitet.</t>
   </si>
   <si>
     <t>Elektromobilität – Autostromvertrag und Ladekarte</t>
@@ -180,6 +169,84 @@
   </si>
   <si>
     <t>Änderungen der Bankverbindung bzw. Bankdaten werden von den Stadtwerken Waiblingen ausschließlich schriftlich entgegengenommen. Eine telefonische Änderung der Bankdaten ist nicht möglich. Kunden können ihre neue Bankverbindung über das entsprechende Formular auf der Website mitteilen oder die Änderung vor Ort im Kundencenter vornehmen.</t>
+  </si>
+  <si>
+    <t>Guthaben - Auszahlung</t>
+  </si>
+  <si>
+    <t>Haben Sie ein Guthaben und noch kein SEPA-Lastschriftmandat bei den Stadtwerken Waiblingen hinterlegt, werden für die Auszahlung die Kontodaten benötigt. Sie müssen hierfür das Guthabenformular auf der Website nutzen oder die Kontodaten per E-Mail an info@stadtwerke-waiblingen.de übermitteln. Nach einer kurzen Prüfung wird die Auszahlung des Guthabens veranlasst.</t>
+  </si>
+  <si>
+    <t>Guthaben - Zeitpunkt Auszahlung</t>
+  </si>
+  <si>
+    <t>Nach einer kurzen Prüfung wird die Auszahlung Ihres Guthabens veranlasst.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Abschaltankündigung</t>
+  </si>
+  <si>
+    <t>Eine Abschaltankündigung sollte ernst genommen und innerhalb der darin genannten Frist bearbeitet werden, um eine Unterbrechung der Energieversorgung zu vermeiden. Der offene Betrag muss bis zu dem in der Abschaltankündigung genannten Termin vollständig beglichen werden.</t>
+  </si>
+  <si>
+    <t>Abschaltung - Zahlungsschwierigkeiten</t>
+  </si>
+  <si>
+    <t>Können Sie den in der Abschaltankündigung genannten offenen Betrag derzeit nicht vollständig bezahlen, sollten Sie sich zeitnah vor Ort an das Kundencenter der Stadtwerke Waiblingen wenden. Dort kann gemeinsam geprüft werden, welche passende Lösung für die offene Forderung möglich ist.</t>
+  </si>
+  <si>
+    <t>Abschaltung - Zahlung bereits erfolgt</t>
+  </si>
+  <si>
+    <t>Haben Sie trotz bereits erfolgter Zahlung eine Abschaltankündigung erhalten, muss zunächst geprüft werden, ob der vollständige offene Betrag auf das richtige Konto der Stadtwerke Waiblingen überwiesen wurde. Sind Bankverbindung und Betrag korrekt, ist das auf der Abschaltankündigung angegebene Datum „Zahlungen berücksichtigt bis“ zu beachten. Ist die Zahlung erst nach diesem Datum bei den Stadtwerken eingegangen, haben sich Zahlung und Abschaltankündigung zeitlich überschnitten und die Abschaltankündigung ist hinfällig. Wenn Sie Fragen hierzu haben, melden Sie sich bitte per E-Mail an info@stadtwerke-waiblingen.de.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Begleichung im Kundencenter</t>
+  </si>
+  <si>
+    <t>Ein aufgrund einer Abschaltung offener Betrag kann direkt im Kundencenter der Stadtwerke Waiblingen beglichen werden. Sobald die offene Forderung vollständig bezahlt ist, wird die Wiederherstellung der Versorgung veranlasst.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Wiederherstellung der Versorgung</t>
+  </si>
+  <si>
+    <t>Nach vollständiger Begleichung der offenen Forderung wird die Wiederherstellung der Energieversorgung umgehend veranlasst. In vielen Fällen kann die Wiederherstellung noch am selben Arbeitstag erfolgen.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Wiederherstellung der Gasversorgung</t>
+  </si>
+  <si>
+    <t>Wurde die Gasversorgung unterbrochen, ist vor der Wiederinbetriebnahme zusätzlich eine gesetzlich vorgeschriebene Druckprüfung erforderlich. Diese Prüfung muss vom Kunden bei einem zugelassenen Installateur beauftragt werden. Erst nach Erfüllung der erforderlichen Voraussetzungen kann die Gasversorgung wiederhergestellt werden.</t>
+  </si>
+  <si>
+    <t>Inkasso – Forderung an externe Kanzlei übergeben</t>
+  </si>
+  <si>
+    <t>Offene Forderungen werden von den Stadtwerken Waiblingen zur weiteren Bearbeitung an externe Kanzleien bzw. Inkassodienstleister übergeben. Dazu gehören E-Rechtsanwälte, On Collect und Dornbach. Bei Fragen zu einem erhaltenen Schreiben, zur Höhe oder zum Grund der Forderung, zu einer früheren Wohnadresse oder zur Echtheit des Schreibens wenden Sie sich bitte direkt an die auf dem Schreiben genannte zuständige Kanzlei bzw. den Inkassodienstleister. Nach Übergabe der Forderung haben die Stadtwerke Waiblingen keinen Einfluss mehr auf die weitere Bearbeitung und können hierzu keine inhaltlichen Auskünfte geben.</t>
+  </si>
+  <si>
+    <t>Mahnung – Zahlung bereits erfolgt oder Rückstand unklar</t>
+  </si>
+  <si>
+    <t>Prüfen Sie bitte zunächst, ob Sie den vollständigen Betrag auf das richtige Konto der Stadtwerke Waiblingen überwiesen haben. Stimmen Bankverbindung und überwiesener Betrag, prüfen Sie bitte anschließend das auf der Mahnung angegebene Datum „Zahlungen berücksichtigt bis“. Ist Ihre Zahlung erst nach diesem Datum eingegangen, haben sich Zahlung und Mahnung zeitlich überschnitten und die Mahnung ist hinfällig. Bei weiteren Fragen oder Unklarheiten können Sie uns gerne per E-Mail an info@stadtwerke-waiblingen.de kontaktieren.</t>
+  </si>
+  <si>
+    <t>Mahnung – Trotz regelmäßiger Abschlagszahlung</t>
+  </si>
+  <si>
+    <t>Prüfen Sie bitte zunächst, ob Sie zwischenzeitlich eine Jahresverbrauchsabrechnung erhalten haben. Aus der Jahresverbrauchsabrechnung kann sich eine Nachzahlung ergeben, die noch offen ist. Außerdem kann mit der Jahresverbrauchsabrechnung Ihr monatlicher Abschlag angepasst bzw. erhöht worden sein. Prüfen Sie daher bitte, ob sich der angemahnte Betrag aus einer offenen Nachzahlung oder einem geänderten Abschlagsbetrag ergibt.</t>
+  </si>
+  <si>
+    <t>Mahnung – Mahngebühren</t>
+  </si>
+  <si>
+    <t>Haben Sie eine Zahlungserinnerung erhalten, fallen dafür keine Mahngebühren an. Haben Sie hingegen eine Mahnung erhalten, werden Mahngebühren in Höhe von 4,00 Euro berechnet. Bitte berücksichtigen Sie die Mahngebühr zusätzlich zum offenen Betrag bei Ihrer Zahlung.</t>
+  </si>
+  <si>
+    <t>Ratenzahlung – Offene Jahresverbrauchsabrechnung</t>
+  </si>
+  <si>
+    <t>Können Sie eine offene Jahresverbrauchsabrechnung nicht auf einmal bezahlen, kann eine Ratenzahlungsvereinbarung mit einer Laufzeit von maximal sechs Monaten beantragt werden. Der Ratenvertrag kann jeweils zum 1. oder zum 15. eines Monats beginnen. Möchten Sie eine Ratenzahlung vereinbaren, senden Sie uns bitte eine E-Mail an info@stadtwerke-waiblingen.de und teilen Sie uns die gewünschten Angaben zur Ratenzahlung mit. Ihr Antrag wird anschließend geprüft. Bei Bewilligung erhalten Sie den Ratenzahlungsvertrag in den nächsten Tagen in Papierform.</t>
   </si>
 </sst>
 </file>
@@ -203,14 +270,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -224,8 +283,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -241,6 +306,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -296,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -308,17 +379,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -633,12 +709,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:D28"/>
+  <dimension ref="B2:D40"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.42578125" customWidth="1"/>
     <col min="2" max="2" width="43.28515625" customWidth="1"/>
-    <col min="3" max="3" width="134.42578125" customWidth="1"/>
+    <col min="3" max="3" width="170.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="23.25" customHeight="1">
@@ -728,59 +804,59 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="75">
-      <c r="B14" s="4" t="s">
+    <row r="14" spans="2:4">
+      <c r="B14" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="60">
-      <c r="B15" s="8" t="s">
+    <row r="15" spans="2:4">
+      <c r="B15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="90">
-      <c r="B16" s="9" t="s">
+    <row r="16" spans="2:4" ht="75">
+      <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="35.25" customHeight="1">
-      <c r="B17" s="3" t="s">
+    <row r="17" spans="2:3" ht="60">
+      <c r="B17" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="30">
-      <c r="B18" s="3" t="s">
+    <row r="18" spans="2:3" ht="90">
+      <c r="B18" s="9" t="s">
         <v>29</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="30">
+    <row r="19" spans="2:3" ht="35.25" customHeight="1">
       <c r="B19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="33.75" customHeight="1">
+    <row r="20" spans="2:3" ht="30">
       <c r="B20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="4" t="s">
         <v>34</v>
       </c>
     </row>
@@ -788,41 +864,149 @@
       <c r="B21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="45">
+    <row r="22" spans="2:3" ht="33.75" customHeight="1">
       <c r="B22" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="2:3">
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-    </row>
-    <row r="24" spans="2:3">
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-    </row>
-    <row r="25" spans="2:3">
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
+    <row r="23" spans="2:3" ht="30">
+      <c r="B23" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" ht="45">
+      <c r="B24" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" ht="45.75">
+      <c r="B25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="26" spans="2:3">
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-    </row>
-    <row r="27" spans="2:3">
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-    </row>
-    <row r="28" spans="2:3">
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+      <c r="B26" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" ht="30">
+      <c r="B27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="45">
+      <c r="B28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="75">
+      <c r="B29" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" ht="30">
+      <c r="B30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="30">
+      <c r="B31" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" ht="45">
+      <c r="B32" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" ht="75">
+      <c r="B33" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" ht="60">
+      <c r="B34" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" ht="48" customHeight="1">
+      <c r="B35" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" ht="30">
+      <c r="B36" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" ht="63.75" customHeight="1">
+      <c r="B37" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+    </row>
+    <row r="39" spans="2:3">
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+    </row>
+    <row r="40" spans="2:3">
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -831,6 +1015,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100C9AF8E73F89E4941919268EDCA0429A4" ma:contentTypeVersion="6" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="c305af0e927197dd7dfb9bc9a29c8323">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e01fda85-2bd3-4106-a425-b6fd761820cd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="925103c6ea15d344ca52a369f48ddba2" ns2:_="">
     <xsd:import namespace="e01fda85-2bd3-4106-a425-b6fd761820cd"/>
@@ -986,23 +1185,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1010,5 +1194,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}"/>
 </file>
</xml_diff>

<commit_message>
update the Excel file(33 rows)
</commit_message>
<xml_diff>
--- a/Excels/Knowledge Base.xlsx
+++ b/Excels/Knowledge Base.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itservicewn.sharepoint.com/sites/VODAFONEVIER/Freigegebene Dokumente/General/FAQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C437004-640A-488E-8379-CFE0609A3568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE63BB4F-29FE-4BDB-B71C-0B8AA884EBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>Zusätzliche Informationen / Wissensdatenbank für den FAQ-Bot</t>
   </si>
@@ -96,30 +96,7 @@
     <t>Einspeiseanlagen – Zählerstand</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Für Einspeiseanlagen ist der Zählerstand mit dem Zählercode </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2.8.0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> relevant. Dieser Wert zeigt die ins Stromnetz eingespeiste Energiemenge an und ist für die Abrechnung der Einspeisevergütung relevant.</t>
-    </r>
+    <t>Für Einspeiseanlagen ist der Zählerstand mit dem Zählercode 2.8.0 relevant. Dieser Wert zeigt die ins Stromnetz eingespeiste Energiemenge an und ist für die Abrechnung der Einspeisevergütung relevant.</t>
   </si>
   <si>
     <t>Freibad Waiblingen – Öffnungszeiten</t>
@@ -128,6 +105,18 @@
     <t>Das Freibad Waiblingen ist jährlich vom 1. Mai bis 15. September geöffnet. Während dieses Zeitraums gelten täglich die Öffnungszeiten von 07:00 Uhr bis 20:00 Uhr.</t>
   </si>
   <si>
+    <t>Freibad Waiblingen - Badeschluss</t>
+  </si>
+  <si>
+    <t>Badeschluss ist im Freibad Waiblingen ist um 19:40 Uhr.</t>
+  </si>
+  <si>
+    <t>Freibad Waiblingen - Ermäßigung Rentner</t>
+  </si>
+  <si>
+    <t>Nein, Rentner erhalten keine Ermäßigung im Freibad Waiblingen.</t>
+  </si>
+  <si>
     <t>Gasversorgung – Belieferung außerhalb des Versorgungsgebiets</t>
   </si>
   <si>
@@ -143,13 +132,13 @@
     <t>Lieferantenwechsel – Widerruf Fremdvertrag</t>
   </si>
   <si>
-    <t>Hat ein Kunde versehentlich oder ungewollt einen Vertrag bei einem anderen Energieversorger abgeschlossen und möchte weiterhin von den Stadtwerken Waiblingen beliefert werden, muss der Vertrag beim anderen Lieferanten widerrufen werden. Dies gilt beispielsweise auch für Verträge, die an der Haustür abgeschlossen wurden oder zu deren Abschluss sich der Kunde überredet fühlte. Für die Prüfung und weitere Bearbeitung durch die Stadtwerke Waiblingen wird die schriftliche Widerrufsbestätigung des anderen Lieferanten benötigt. Der Kunde soll diese Bestätigung per E-Mail an Vertrieb@stadtwerke-waiblingen.de senden. Nach Eingang der Widerrufsbestätigung wird der Vorgang geprüft und bearbeitet.</t>
+    <t>Haben Sie versehentlich oder ungewollt einen Vertrag bei einem anderen Energieversorger abgeschlossen und möchten weiterhin von den Stadtwerken Waiblingen beliefert werden, muss der Vertrag beim anderen Lieferanten widerrufen werden. Dies gilt beispielsweise auch für Verträge, die an der Haustür abgeschlossen wurden oder zu deren Abschluss sich der Kunde überredet fühlte. Für die Prüfung und weitere Bearbeitung durch die Stadtwerke Waiblingen wird die schriftliche Widerrufsbestätigung des anderen Lieferanten benötigt. Der Kunde soll diese Bestätigung per E-Mail an Vertrieb@stadtwerke-waiblingen.de senden. Nach Eingang der Widerrufsbestätigung wird der Vorgang geprüft und bearbeitet.</t>
   </si>
   <si>
     <t>Tarifwechsel – Widerruf</t>
   </si>
   <si>
-    <t>Ein bereits angestoßener Tarifwechsel kann widerrufen werden. Der Widerruf muss schriftlich erfolgen. Hierfür kann der Kunde eine E-Mail an den Vertrieb der Stadtwerke Waiblingen senden oder den Widerrufs-Button auf der Website nutzen. Nach Eingang des Widerrufs wird das Anliegen geprüft und bearbeitet.</t>
+    <t>Ein bereits angestoßener Tarifwechsel kann widerrufen werden. Der Widerruf muss schriftlich erfolgen. Hierfür können Sie eine E-Mail an vertrieb@stadtwerke-waiblingen.de senden oder den Widerrufs-Button auf der Website nutzen. Nach Eingang des Widerrufs wird das Anliegen geprüft und bearbeitet.</t>
   </si>
   <si>
     <t>Elektromobilität – Autostromvertrag und Ladekarte</t>
@@ -180,6 +169,84 @@
   </si>
   <si>
     <t>Änderungen der Bankverbindung bzw. Bankdaten werden von den Stadtwerken Waiblingen ausschließlich schriftlich entgegengenommen. Eine telefonische Änderung der Bankdaten ist nicht möglich. Kunden können ihre neue Bankverbindung über das entsprechende Formular auf der Website mitteilen oder die Änderung vor Ort im Kundencenter vornehmen.</t>
+  </si>
+  <si>
+    <t>Guthaben - Auszahlung</t>
+  </si>
+  <si>
+    <t>Haben Sie ein Guthaben und noch kein SEPA-Lastschriftmandat bei den Stadtwerken Waiblingen hinterlegt, werden für die Auszahlung die Kontodaten benötigt. Sie müssen hierfür das Guthabenformular auf der Website nutzen oder die Kontodaten per E-Mail an info@stadtwerke-waiblingen.de übermitteln. Nach einer kurzen Prüfung wird die Auszahlung des Guthabens veranlasst.</t>
+  </si>
+  <si>
+    <t>Guthaben - Zeitpunkt Auszahlung</t>
+  </si>
+  <si>
+    <t>Nach einer kurzen Prüfung wird die Auszahlung Ihres Guthabens veranlasst.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Abschaltankündigung</t>
+  </si>
+  <si>
+    <t>Eine Abschaltankündigung sollte ernst genommen und innerhalb der darin genannten Frist bearbeitet werden, um eine Unterbrechung der Energieversorgung zu vermeiden. Der offene Betrag muss bis zu dem in der Abschaltankündigung genannten Termin vollständig beglichen werden.</t>
+  </si>
+  <si>
+    <t>Abschaltung - Zahlungsschwierigkeiten</t>
+  </si>
+  <si>
+    <t>Können Sie den in der Abschaltankündigung genannten offenen Betrag derzeit nicht vollständig bezahlen, sollten Sie sich zeitnah vor Ort an das Kundencenter der Stadtwerke Waiblingen wenden. Dort kann gemeinsam geprüft werden, welche passende Lösung für die offene Forderung möglich ist.</t>
+  </si>
+  <si>
+    <t>Abschaltung - Zahlung bereits erfolgt</t>
+  </si>
+  <si>
+    <t>Haben Sie trotz bereits erfolgter Zahlung eine Abschaltankündigung erhalten, muss zunächst geprüft werden, ob der vollständige offene Betrag auf das richtige Konto der Stadtwerke Waiblingen überwiesen wurde. Sind Bankverbindung und Betrag korrekt, ist das auf der Abschaltankündigung angegebene Datum „Zahlungen berücksichtigt bis“ zu beachten. Ist die Zahlung erst nach diesem Datum bei den Stadtwerken eingegangen, haben sich Zahlung und Abschaltankündigung zeitlich überschnitten und die Abschaltankündigung ist hinfällig. Wenn Sie Fragen hierzu haben, melden Sie sich bitte per E-Mail an info@stadtwerke-waiblingen.de.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Begleichung im Kundencenter</t>
+  </si>
+  <si>
+    <t>Ein aufgrund einer Abschaltung offener Betrag kann direkt im Kundencenter der Stadtwerke Waiblingen beglichen werden. Sobald die offene Forderung vollständig bezahlt ist, wird die Wiederherstellung der Versorgung veranlasst.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Wiederherstellung der Versorgung</t>
+  </si>
+  <si>
+    <t>Nach vollständiger Begleichung der offenen Forderung wird die Wiederherstellung der Energieversorgung umgehend veranlasst. In vielen Fällen kann die Wiederherstellung noch am selben Arbeitstag erfolgen.</t>
+  </si>
+  <si>
+    <t>Abschaltung – Wiederherstellung der Gasversorgung</t>
+  </si>
+  <si>
+    <t>Wurde die Gasversorgung unterbrochen, ist vor der Wiederinbetriebnahme zusätzlich eine gesetzlich vorgeschriebene Druckprüfung erforderlich. Diese Prüfung muss vom Kunden bei einem zugelassenen Installateur beauftragt werden. Erst nach Erfüllung der erforderlichen Voraussetzungen kann die Gasversorgung wiederhergestellt werden.</t>
+  </si>
+  <si>
+    <t>Inkasso – Forderung an externe Kanzlei übergeben</t>
+  </si>
+  <si>
+    <t>Offene Forderungen werden von den Stadtwerken Waiblingen zur weiteren Bearbeitung an externe Kanzleien bzw. Inkassodienstleister übergeben. Dazu gehören E-Rechtsanwälte, On Collect und Dornbach. Bei Fragen zu einem erhaltenen Schreiben, zur Höhe oder zum Grund der Forderung, zu einer früheren Wohnadresse oder zur Echtheit des Schreibens wenden Sie sich bitte direkt an die auf dem Schreiben genannte zuständige Kanzlei bzw. den Inkassodienstleister. Nach Übergabe der Forderung haben die Stadtwerke Waiblingen keinen Einfluss mehr auf die weitere Bearbeitung und können hierzu keine inhaltlichen Auskünfte geben.</t>
+  </si>
+  <si>
+    <t>Mahnung – Zahlung bereits erfolgt oder Rückstand unklar</t>
+  </si>
+  <si>
+    <t>Prüfen Sie bitte zunächst, ob Sie den vollständigen Betrag auf das richtige Konto der Stadtwerke Waiblingen überwiesen haben. Stimmen Bankverbindung und überwiesener Betrag, prüfen Sie bitte anschließend das auf der Mahnung angegebene Datum „Zahlungen berücksichtigt bis“. Ist Ihre Zahlung erst nach diesem Datum eingegangen, haben sich Zahlung und Mahnung zeitlich überschnitten und die Mahnung ist hinfällig. Bei weiteren Fragen oder Unklarheiten können Sie uns gerne per E-Mail an info@stadtwerke-waiblingen.de kontaktieren.</t>
+  </si>
+  <si>
+    <t>Mahnung – Trotz regelmäßiger Abschlagszahlung</t>
+  </si>
+  <si>
+    <t>Prüfen Sie bitte zunächst, ob Sie zwischenzeitlich eine Jahresverbrauchsabrechnung erhalten haben. Aus der Jahresverbrauchsabrechnung kann sich eine Nachzahlung ergeben, die noch offen ist. Außerdem kann mit der Jahresverbrauchsabrechnung Ihr monatlicher Abschlag angepasst bzw. erhöht worden sein. Prüfen Sie daher bitte, ob sich der angemahnte Betrag aus einer offenen Nachzahlung oder einem geänderten Abschlagsbetrag ergibt.</t>
+  </si>
+  <si>
+    <t>Mahnung – Mahngebühren</t>
+  </si>
+  <si>
+    <t>Haben Sie eine Zahlungserinnerung erhalten, fallen dafür keine Mahngebühren an. Haben Sie hingegen eine Mahnung erhalten, werden Mahngebühren in Höhe von 4,00 Euro berechnet. Bitte berücksichtigen Sie die Mahngebühr zusätzlich zum offenen Betrag bei Ihrer Zahlung.</t>
+  </si>
+  <si>
+    <t>Ratenzahlung – Offene Jahresverbrauchsabrechnung</t>
+  </si>
+  <si>
+    <t>Können Sie eine offene Jahresverbrauchsabrechnung nicht auf einmal bezahlen, kann eine Ratenzahlungsvereinbarung mit einer Laufzeit von maximal sechs Monaten beantragt werden. Der Ratenvertrag kann jeweils zum 1. oder zum 15. eines Monats beginnen. Möchten Sie eine Ratenzahlung vereinbaren, senden Sie uns bitte eine E-Mail an info@stadtwerke-waiblingen.de und teilen Sie uns die gewünschten Angaben zur Ratenzahlung mit. Ihr Antrag wird anschließend geprüft. Bei Bewilligung erhalten Sie den Ratenzahlungsvertrag in den nächsten Tagen in Papierform.</t>
   </si>
 </sst>
 </file>
@@ -203,14 +270,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -224,8 +283,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -241,6 +306,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -296,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -308,17 +379,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -633,12 +709,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:D28"/>
+  <dimension ref="B2:D40"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.42578125" customWidth="1"/>
     <col min="2" max="2" width="43.28515625" customWidth="1"/>
-    <col min="3" max="3" width="134.42578125" customWidth="1"/>
+    <col min="3" max="3" width="170.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="23.25" customHeight="1">
@@ -728,59 +804,59 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="75">
-      <c r="B14" s="4" t="s">
+    <row r="14" spans="2:4">
+      <c r="B14" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="60">
-      <c r="B15" s="8" t="s">
+    <row r="15" spans="2:4">
+      <c r="B15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="90">
-      <c r="B16" s="9" t="s">
+    <row r="16" spans="2:4" ht="75">
+      <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="35.25" customHeight="1">
-      <c r="B17" s="3" t="s">
+    <row r="17" spans="2:3" ht="60">
+      <c r="B17" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="30">
-      <c r="B18" s="3" t="s">
+    <row r="18" spans="2:3" ht="90">
+      <c r="B18" s="9" t="s">
         <v>29</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="30">
+    <row r="19" spans="2:3" ht="35.25" customHeight="1">
       <c r="B19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="33.75" customHeight="1">
+    <row r="20" spans="2:3" ht="30">
       <c r="B20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="4" t="s">
         <v>34</v>
       </c>
     </row>
@@ -788,41 +864,149 @@
       <c r="B21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="45">
+    <row r="22" spans="2:3" ht="33.75" customHeight="1">
       <c r="B22" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="2:3">
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-    </row>
-    <row r="24" spans="2:3">
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-    </row>
-    <row r="25" spans="2:3">
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
+    <row r="23" spans="2:3" ht="30">
+      <c r="B23" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" ht="45">
+      <c r="B24" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" ht="45.75">
+      <c r="B25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="26" spans="2:3">
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-    </row>
-    <row r="27" spans="2:3">
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-    </row>
-    <row r="28" spans="2:3">
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+      <c r="B26" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" ht="30">
+      <c r="B27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="45">
+      <c r="B28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="75">
+      <c r="B29" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" ht="30">
+      <c r="B30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="30">
+      <c r="B31" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" ht="45">
+      <c r="B32" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" ht="75">
+      <c r="B33" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" ht="60">
+      <c r="B34" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" ht="48" customHeight="1">
+      <c r="B35" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" ht="30">
+      <c r="B36" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" ht="63.75" customHeight="1">
+      <c r="B37" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+    </row>
+    <row r="39" spans="2:3">
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+    </row>
+    <row r="40" spans="2:3">
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -831,6 +1015,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100C9AF8E73F89E4941919268EDCA0429A4" ma:contentTypeVersion="6" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="c305af0e927197dd7dfb9bc9a29c8323">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e01fda85-2bd3-4106-a425-b6fd761820cd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="925103c6ea15d344ca52a369f48ddba2" ns2:_="">
     <xsd:import namespace="e01fda85-2bd3-4106-a425-b6fd761820cd"/>
@@ -986,23 +1185,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1010,5 +1194,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{552932D6-818C-4E5F-A4DC-6AD4FB3E74DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{891F6E60-2DC7-4183-8443-781947774D29}"/>
 </file>
</xml_diff>